<commit_message>
feat: add route editing and shipment management features to frontend
</commit_message>
<xml_diff>
--- a/public/rh-imports/employees-only-sample.xlsx
+++ b/public/rh-imports/employees-only-sample.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Importacao" sheetId="1" r:id="rId1"/>
+    <sheet name="Funcionarios" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,116 +397,331 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:Z4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>nome</v>
+      </c>
+      <c r="B1" t="str">
         <v>email</v>
-      </c>
-      <c r="B1" t="str">
-        <v>name</v>
       </c>
       <c r="C1" t="str">
         <v>cpf</v>
       </c>
       <c r="D1" t="str">
-        <v>role</v>
+        <v>perfil</v>
       </c>
       <c r="E1" t="str">
-        <v>status</v>
+        <v>filial</v>
       </c>
       <c r="F1" t="str">
-        <v>branchName</v>
+        <v>departamento</v>
       </c>
       <c r="G1" t="str">
-        <v>departmentName</v>
+        <v>cargo</v>
       </c>
       <c r="H1" t="str">
-        <v>admissionDate</v>
+        <v>matricula</v>
       </c>
       <c r="I1" t="str">
-        <v>registration</v>
+        <v>situacao</v>
       </c>
       <c r="J1" t="str">
-        <v>currentSalary</v>
+        <v>dataAdmissao</v>
       </c>
       <c r="K1" t="str">
-        <v>directManagerEmail</v>
+        <v>dataDemissao</v>
+      </c>
+      <c r="L1" t="str">
+        <v>dataNascimento</v>
+      </c>
+      <c r="M1" t="str">
+        <v>salarioAtual</v>
+      </c>
+      <c r="N1" t="str">
+        <v>emailGestorDireto</v>
+      </c>
+      <c r="O1" t="str">
+        <v>sexo</v>
+      </c>
+      <c r="P1" t="str">
+        <v>rg</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>ctps</v>
+      </c>
+      <c r="R1" t="str">
+        <v>cnh</v>
+      </c>
+      <c r="S1" t="str">
+        <v>escolaridade</v>
+      </c>
+      <c r="T1" t="str">
+        <v>nomeDaMae</v>
+      </c>
+      <c r="U1" t="str">
+        <v>nomeDoPai</v>
+      </c>
+      <c r="V1" t="str">
+        <v>endereco</v>
+      </c>
+      <c r="W1" t="str">
+        <v>cidade</v>
+      </c>
+      <c r="X1" t="str">
+        <v>uf</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>nomeDoConjuge</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>telefoneConjuge</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>João da Silva</v>
+      </c>
+      <c r="B2" t="str">
         <v>joao.silva@toclog.com.br</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Joao da Silva</v>
       </c>
       <c r="C2" t="str">
         <v>12345678911</v>
       </c>
       <c r="D2" t="str">
+        <v>USER</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Matriz - São Paulo</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Recursos Humanos</v>
+      </c>
+      <c r="G2" t="str">
         <v>Analista de RH</v>
       </c>
-      <c r="E2" t="str">
+      <c r="H2" t="str">
+        <v>RH-001</v>
+      </c>
+      <c r="I2" t="str">
         <v>ACTIVE</v>
       </c>
-      <c r="F2" t="str">
-        <v>Matriz - São Paulo</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Recursos Humanos</v>
-      </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>2026-01-10</v>
       </c>
-      <c r="I2" t="str">
-        <v>RH-001</v>
-      </c>
-      <c r="J2" t="str">
-        <v>4500.00</v>
-      </c>
       <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v>1992-04-18</v>
+      </c>
+      <c r="M2">
+        <v>4500</v>
+      </c>
+      <c r="N2" t="str">
         <v>ana.rh@toclog.com.br</v>
+      </c>
+      <c r="O2" t="str">
+        <v>MASCULINO</v>
+      </c>
+      <c r="P2" t="str">
+        <v>12.345.678-9</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>1234567/001-SP</v>
+      </c>
+      <c r="R2" t="str">
+        <v>12345678900</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Superior Completo</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Maria Aparecida da Silva</v>
+      </c>
+      <c r="U2" t="str">
+        <v>José da Silva</v>
+      </c>
+      <c r="V2" t="str">
+        <v>Av. Paulista, 1000, Apto 42</v>
+      </c>
+      <c r="W2" t="str">
+        <v>São Paulo</v>
+      </c>
+      <c r="X2" t="str">
+        <v>SP</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>Carla Silva</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>(11) 98765-4321</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>Maria Oliveira</v>
+      </c>
+      <c r="B3" t="str">
         <v>maria.oliveira@toclog.com.br</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Maria Oliveira</v>
       </c>
       <c r="C3" t="str">
         <v>12345678912</v>
       </c>
       <c r="D3" t="str">
+        <v>USER</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Filial - Rio de Janeiro</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="G3" t="str">
         <v>Assistente de Compras</v>
       </c>
-      <c r="E3" t="str">
+      <c r="H3" t="str">
+        <v>CMP-014</v>
+      </c>
+      <c r="I3" t="str">
         <v>ACTIVE</v>
       </c>
-      <c r="F3" t="str">
-        <v>Filial - Rio de Janeiro</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Compras</v>
-      </c>
-      <c r="H3" t="str">
+      <c r="J3" t="str">
         <v>2026-02-15</v>
       </c>
-      <c r="I3" t="str">
-        <v>CMP-014</v>
-      </c>
-      <c r="J3" t="str">
-        <v>3200.00</v>
-      </c>
       <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v>1995-11-23</v>
+      </c>
+      <c r="M3">
+        <v>3200</v>
+      </c>
+      <c r="N3" t="str">
         <v>carlos.compras@toclog.com.br</v>
+      </c>
+      <c r="O3" t="str">
+        <v>FEMININO</v>
+      </c>
+      <c r="P3" t="str">
+        <v>23.456.789-0</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>7654321/002-RJ</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v>Superior Incompleto</v>
+      </c>
+      <c r="T3" t="str">
+        <v>Sandra Regina Oliveira</v>
+      </c>
+      <c r="U3" t="str">
+        <v>Antônio Oliveira</v>
+      </c>
+      <c r="V3" t="str">
+        <v>Rua das Laranjeiras, 250</v>
+      </c>
+      <c r="W3" t="str">
+        <v>Rio de Janeiro</v>
+      </c>
+      <c r="X3" t="str">
+        <v>RJ</v>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Carlos Eduardo Santos</v>
+      </c>
+      <c r="B4" t="str">
+        <v>carlos.santos@toclog.com.br</v>
+      </c>
+      <c r="C4" t="str">
+        <v>12345678913</v>
+      </c>
+      <c r="D4" t="str">
+        <v>RH_MANAGER</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Matriz - São Paulo</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Recursos Humanos</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Coordenador de RH</v>
+      </c>
+      <c r="H4" t="str">
+        <v>RH-002</v>
+      </c>
+      <c r="I4" t="str">
+        <v>ACTIVE</v>
+      </c>
+      <c r="J4" t="str">
+        <v>2025-08-01</v>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v>1988-03-05</v>
+      </c>
+      <c r="M4">
+        <v>7800</v>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v>MASCULINO</v>
+      </c>
+      <c r="P4" t="str">
+        <v>34.567.890-1</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>9876543/001-SP</v>
+      </c>
+      <c r="R4" t="str">
+        <v>98765432100</v>
+      </c>
+      <c r="S4" t="str">
+        <v>Pós-graduação</v>
+      </c>
+      <c r="T4" t="str">
+        <v>Helena Santos</v>
+      </c>
+      <c r="U4" t="str">
+        <v>Paulo Roberto Santos</v>
+      </c>
+      <c r="V4" t="str">
+        <v>Rua Augusta, 500</v>
+      </c>
+      <c r="W4" t="str">
+        <v>São Paulo</v>
+      </c>
+      <c r="X4" t="str">
+        <v>SP</v>
+      </c>
+      <c r="Y4" t="str">
+        <v>Patrícia Santos</v>
+      </c>
+      <c r="Z4" t="str">
+        <v>(11) 91234-5678</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>